<commit_message>
feat: agregar Dimension 5 (Caso de Uso y Viabilidad) al instrumento AI-DLC - Nueva dimension con 5 preguntas de viabilidad tecnica y caso concreto - Prompt IA: agregar Regla 3 (senal de viabilidad) para interpretar eje bajo - Prompt optimizado y compactado para caber en 6000 chars - Subir limite de sanitizacion a 6000 - Regenerar Excel con 5 dimensiones y 22 preguntas
</commit_message>
<xml_diff>
--- a/docs/diagnostico-preparacion-aidlc.xlsx
+++ b/docs/diagnostico-preparacion-aidlc.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="65">
   <si>
     <t>Dimensión</t>
   </si>
@@ -118,6 +118,30 @@
   </si>
   <si>
     <t>Operamos en un sector con exigencias de cumplimiento o gobernanza que el software debe satisfacer.</t>
+  </si>
+  <si>
+    <t>Caso de Uso y Viabilidad</t>
+  </si>
+  <si>
+    <t>Evalúa si existe un caso de uso concreto identificado y las condiciones técnicas mínimas para ejecutarlo.</t>
+  </si>
+  <si>
+    <t>#E85D04</t>
+  </si>
+  <si>
+    <t>Tenemos identificado al menos un caso de uso concreto que queremos llevar a producción con AI-DLC.</t>
+  </si>
+  <si>
+    <t>El caso de uso tiene un dueño de negocio que puede definir criterios de aceptación.</t>
+  </si>
+  <si>
+    <t>Conocemos las restricciones regulatorias o de seguridad que el caso debe cumplir.</t>
+  </si>
+  <si>
+    <t>Contamos con infraestructura cloud (AWS u otra) disponible para soportar el desarrollo.</t>
+  </si>
+  <si>
+    <t>Podemos proveer acceso a herramientas de desarrollo modernas (IDE, repositorios, CI/CD) sin restricciones corporativas bloqueantes.</t>
   </si>
   <si>
     <t>Valor</t>
@@ -564,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -932,6 +956,106 @@
         <v>34</v>
       </c>
       <c r="F18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22">
+        <v>5</v>
+      </c>
+      <c r="E22" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23">
+        <v>5</v>
+      </c>
+      <c r="E23" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23">
         <v>5</v>
       </c>
     </row>
@@ -953,13 +1077,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -967,10 +1091,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -978,10 +1102,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -989,10 +1113,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1000,10 +1124,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1011,10 +1135,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1035,24 +1159,24 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -1063,7 +1187,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -1077,7 +1201,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
@@ -1091,10 +1215,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C5">
         <v>4.5</v>

</xml_diff>

<commit_message>
Feature/multi instrument vision (#29)
* excel

* fix: actualizar metadata OG del portal (titulo y descripcion)

* feat: metadata dinamica en URL de encuesta segun instrumento y sesion

* docs: actualizar README y manual de administrador con ultimas features

* docs: actualizar roadmap - priorizar admin de usuarios y roles

* fix: hacer panel admin responsive para mobile

* security: corregir 5 vulnerabilidades criticas identificadas en code review

* perf+security: fixes de nivel medio del code review

* a11y+quality: focus trap en modales, aria-labels en escala, eliminar import deprecado

* feat: tracking de consumo por usuario - sesiones, analisis IA y tokens por modelo

* ci: actualizar actions a v5 y Node.js 22 (fix deprecation Node 20)

* ci: agregar FORCE_JAVASCRIPT_ACTIONS_TO_NODE24 para compatibilidad inmediata

* fix: migrar middleware.ts a proxy.ts (Next.js 16) + quitar node:async_hooks del logger
</commit_message>
<xml_diff>
--- a/docs/diagnostico-preparacion-aidlc.xlsx
+++ b/docs/diagnostico-preparacion-aidlc.xlsx
@@ -1,12 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F38070-360A-4E49-AAC9-164D09366973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Banco de Preguntas" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Escala" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Niveles" state="visible" r:id="rId6"/>
+    <sheet name="Banco de Preguntas" sheetId="1" r:id="rId1"/>
+    <sheet name="Escala" sheetId="2" r:id="rId2"/>
+    <sheet name="Niveles" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -213,17 +217,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -587,9 +593,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
@@ -599,7 +605,7 @@
     <col min="6" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -619,7 +625,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -639,7 +645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -659,7 +665,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -679,7 +685,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -699,7 +705,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -719,7 +725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -739,7 +745,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -759,7 +765,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -779,7 +785,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -799,7 +805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -819,7 +825,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -839,7 +845,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -859,7 +865,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -879,7 +885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -899,7 +905,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -919,7 +925,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -939,7 +945,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -959,7 +965,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -979,7 +985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -999,7 +1005,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -1019,7 +1025,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1039,7 +1045,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -1061,21 +1067,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -1086,7 +1092,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1097,7 +1103,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1108,7 +1114,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1119,7 +1125,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1130,7 +1136,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1143,21 +1149,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -1171,7 +1177,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>59</v>
       </c>
@@ -1185,7 +1191,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>61</v>
       </c>
@@ -1199,7 +1205,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1210,10 +1216,10 @@
         <v>3.5</v>
       </c>
       <c r="D4">
-        <v>4.4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1229,6 +1235,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>